<commit_message>
Update test case report
</commit_message>
<xml_diff>
--- a/Báo cáo test case.xlsx
+++ b/Báo cáo test case.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000" activeTab="9"/>
+    <workbookView windowWidth="23040" windowHeight="9000" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="923" uniqueCount="646">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="925" uniqueCount="647">
   <si>
     <t>TEST CASE</t>
   </si>
@@ -1368,7 +1368,7 @@
     <t>GET /api/promotions?amount=-1</t>
   </si>
   <si>
-    <t>Giá trị amount không hợp lệ phải được xử lý rõ ràng hoặc không trả dữ liệu mặc định như request hợp lệ</t>
+    <t>Trả 400 Bad Request với lỗi “Giá trị đơn hàng không hợp lệ!”</t>
   </si>
   <si>
     <t>TCAPIPro4.png</t>
@@ -1392,7 +1392,7 @@
     <t>TCAPIPro5.png</t>
   </si>
   <si>
-    <t>GET promotion với amount không hợp lệ vẫn xử lý(#Issue 28)</t>
+    <t>GET promotion với amount không hợp lệ vẫn xử lý (#Issue 28). Có thể kiểm tra thêm các giá trị tương đương: amount=ABC, amount=10abc, amount=@@</t>
   </si>
   <si>
     <t>TCAPIPro5SauRetest.png</t>
@@ -1401,7 +1401,7 @@
     <t>TC-API-006</t>
   </si>
   <si>
-    <t>GET promotion theo type không hợp lệ</t>
+    <t>GET promotion theo ptype không hợp lệ</t>
   </si>
   <si>
     <t>GET /api/promotions?ptype=ABC</t>
@@ -1419,7 +1419,7 @@
     <t>TC-API-007</t>
   </si>
   <si>
-    <t>GET promotion theo type hợp lệ</t>
+    <t>GET promotion theo ptype hợp lệ</t>
   </si>
   <si>
     <t>GET /api/promotions?ptype=VOUCHER</t>
@@ -1443,7 +1443,7 @@
     <t>GET /api/promotions?page=0</t>
   </si>
   <si>
-    <t>Giá trị page không hợp lệ phải được xử lý rõ ràng, không nên trả như request hợp lệ</t>
+    <t>Trả 400 Bad Request với lỗi “Số trang không hợp lệ!”</t>
   </si>
   <si>
     <t>TCAPIPro8.png</t>
@@ -1464,9 +1464,6 @@
     <t>GET /api/promotions?page=-1</t>
   </si>
   <si>
-    <t>Giá trị page âm phải được xử lý rõ ràng, không nên trả như request hợp lệ</t>
-  </si>
-  <si>
     <t>TCAPIPro9.png</t>
   </si>
   <si>
@@ -1479,13 +1476,19 @@
     <t>TC-API-010</t>
   </si>
   <si>
+    <t>GET promotion phân trang với page không hợp lệ</t>
+  </si>
+  <si>
     <t>GET /api/promotions?page=abc</t>
   </si>
   <si>
     <t>TCAPIPro10.png</t>
   </si>
   <si>
-    <t>GET promotion với page không hợp lệ chưa được validate (#Issue 29)</t>
+    <t>GET promotion với page không hợp lệ chưa được validate (#Issue 29). Có thể kiểm tra thêm các giá trị tương đương: page=ABC, page=10abc, page=@@</t>
+  </si>
+  <si>
+    <t>TCAPIPro10SauRetest.png</t>
   </si>
   <si>
     <t>2. Kiểm tra POST tạo promotion</t>
@@ -3989,7 +3992,7 @@
   <sheetData>
     <row r="1" customHeight="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="3"/>
@@ -4010,10 +4013,10 @@
     <row r="3" customHeight="1" spans="1:7">
       <c r="A3" s="4"/>
       <c r="B3" s="3" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
@@ -4023,7 +4026,7 @@
     <row r="4" customHeight="1" spans="1:7">
       <c r="A4" s="4"/>
       <c r="B4" s="3" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="C4" s="5">
         <v>46162</v>
@@ -4054,10 +4057,10 @@
     <row r="7" customHeight="1" spans="1:7">
       <c r="A7" s="3"/>
       <c r="B7" s="6" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>48</v>
@@ -4069,7 +4072,7 @@
         <v>49</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
     </row>
     <row r="8" customHeight="1" spans="1:7">
@@ -4078,7 +4081,7 @@
         <v>1</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="D8" s="11">
         <v>8</v>
@@ -4099,7 +4102,7 @@
         <v>2</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="D9" s="10">
         <v>8</v>
@@ -4120,7 +4123,7 @@
         <v>3</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="D10" s="12">
         <v>5</v>
@@ -4141,7 +4144,7 @@
         <v>4</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="D11" s="12">
         <v>4</v>
@@ -4162,7 +4165,7 @@
         <v>5</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="D12" s="12">
         <v>7</v>
@@ -4204,7 +4207,7 @@
         <v>7</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="D14" s="12">
         <v>10</v>
@@ -4225,7 +4228,7 @@
         <v>8</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="D15" s="12">
         <v>16</v>
@@ -4244,7 +4247,7 @@
       <c r="A16" s="3"/>
       <c r="B16" s="13"/>
       <c r="C16" s="14" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="D16" s="15">
         <f>D8+D9+D10+D11+D12+D13+D14+D15</f>
@@ -4275,7 +4278,7 @@
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="D18" s="3"/>
       <c r="E18" s="17">
@@ -4283,7 +4286,7 @@
         <v>100</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="G18" s="10"/>
     </row>
@@ -4291,7 +4294,7 @@
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="D19" s="3"/>
       <c r="E19" s="17">
@@ -4299,7 +4302,7 @@
         <v>76.1363636363636</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="G19" s="10"/>
     </row>
@@ -4970,7 +4973,7 @@
   <cols>
     <col min="1" max="1" width="13.5" customWidth="1"/>
     <col min="2" max="2" width="42.25" customWidth="1"/>
-    <col min="3" max="3" width="86.1111111111111" customWidth="1"/>
+    <col min="3" max="3" width="76.5" customWidth="1"/>
     <col min="6" max="6" width="46" customWidth="1"/>
     <col min="7" max="7" width="33.5" customWidth="1"/>
     <col min="10" max="10" width="30.6296296296296" customWidth="1"/>
@@ -5060,7 +5063,9 @@
       <c r="C6" s="32" t="s">
         <v>49</v>
       </c>
-      <c r="D6" s="32"/>
+      <c r="D6" s="32">
+        <v>0</v>
+      </c>
       <c r="E6" s="28"/>
       <c r="F6" s="28"/>
       <c r="G6" s="28"/>
@@ -5512,7 +5517,7 @@
   <sheetFormatPr defaultColWidth="12.6296296296296" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="2" max="2" width="41.5" customWidth="1"/>
-    <col min="3" max="3" width="68.6666666666667" customWidth="1"/>
+    <col min="3" max="3" width="64" customWidth="1"/>
     <col min="6" max="6" width="43.6296296296296" customWidth="1"/>
     <col min="7" max="7" width="30.6296296296296" customWidth="1"/>
     <col min="10" max="10" width="53.75" customWidth="1"/>
@@ -5962,7 +5967,7 @@
   <dimension ref="A1:L31"/>
   <sheetFormatPr defaultColWidth="12.6296296296296" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="2" max="2" width="63.3333333333333" customWidth="1"/>
+    <col min="2" max="2" width="56.6296296296296" customWidth="1"/>
     <col min="3" max="3" width="98.1296296296296" customWidth="1"/>
     <col min="6" max="6" width="35.75" customWidth="1"/>
     <col min="7" max="7" width="16.8796296296296" customWidth="1"/>
@@ -35326,15 +35331,15 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr defaultColWidth="12.6296296296296" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
-    <col min="2" max="2" width="35.1296296296296" customWidth="1"/>
+    <col min="2" max="2" width="39.3796296296296" customWidth="1"/>
     <col min="3" max="3" width="60.1296296296296" customWidth="1"/>
     <col min="6" max="6" width="57.8796296296296" customWidth="1"/>
     <col min="7" max="7" width="18.1296296296296" customWidth="1"/>
-    <col min="10" max="10" width="54" customWidth="1"/>
+    <col min="10" max="10" width="116.37962962963" customWidth="1"/>
     <col min="11" max="11" width="16.5" customWidth="1"/>
     <col min="12" max="12" width="27" customWidth="1"/>
   </cols>
@@ -35806,12 +35811,12 @@
         <v>474</v>
       </c>
       <c r="D21" s="55" t="s">
-        <v>475</v>
+        <v>468</v>
       </c>
       <c r="E21" s="35"/>
       <c r="F21" s="35"/>
       <c r="G21" s="48" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="H21" s="49">
         <v>46134</v>
@@ -35820,21 +35825,21 @@
         <v>50</v>
       </c>
       <c r="J21" s="50" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="K21" s="50" t="s">
         <v>48</v>
       </c>
       <c r="L21" s="48" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="22" customHeight="1" spans="1:12">
       <c r="A22" s="50" t="s">
+        <v>478</v>
+      </c>
+      <c r="B22" s="54" t="s">
         <v>479</v>
-      </c>
-      <c r="B22" s="54" t="s">
-        <v>473</v>
       </c>
       <c r="C22" s="50" t="s">
         <v>480</v>
@@ -35856,12 +35861,16 @@
       <c r="J22" s="50" t="s">
         <v>482</v>
       </c>
-      <c r="K22" s="50"/>
-      <c r="L22" s="50"/>
+      <c r="K22" s="50" t="s">
+        <v>48</v>
+      </c>
+      <c r="L22" s="48" t="s">
+        <v>483</v>
+      </c>
     </row>
     <row r="23" customHeight="1" spans="1:12">
       <c r="A23" s="44" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B23" s="25"/>
       <c r="C23" s="25"/>
@@ -35877,21 +35886,21 @@
     </row>
     <row r="24" customHeight="1" spans="1:12">
       <c r="A24" s="45" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="B24" s="45" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="C24" s="45" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="D24" s="46" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="E24" s="47"/>
       <c r="F24" s="47"/>
       <c r="G24" s="58" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="H24" s="49">
         <v>46151</v>
@@ -35900,28 +35909,28 @@
         <v>48</v>
       </c>
       <c r="J24" s="45" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="K24" s="45"/>
       <c r="L24" s="45"/>
     </row>
     <row r="25" customHeight="1" spans="1:12">
       <c r="A25" s="45" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="B25" s="45" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="C25" s="45" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="D25" s="46" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="E25" s="47"/>
       <c r="F25" s="47"/>
       <c r="G25" s="58" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="H25" s="49">
         <v>46151</v>
@@ -35930,28 +35939,28 @@
         <v>48</v>
       </c>
       <c r="J25" s="45" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="K25" s="45"/>
       <c r="L25" s="45"/>
     </row>
     <row r="26" customHeight="1" spans="1:12">
       <c r="A26" s="45" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="B26" s="45" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="C26" s="45" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="D26" s="46" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="E26" s="47"/>
       <c r="F26" s="47"/>
       <c r="G26" s="58" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="H26" s="49">
         <v>46151</v>
@@ -35960,28 +35969,28 @@
         <v>48</v>
       </c>
       <c r="J26" s="45" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="K26" s="45"/>
       <c r="L26" s="45"/>
     </row>
     <row r="27" customHeight="1" spans="1:12">
       <c r="A27" s="45" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="B27" s="45" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="C27" s="45" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="D27" s="46" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="E27" s="47"/>
       <c r="F27" s="47"/>
       <c r="G27" s="58" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="H27" s="49">
         <v>46151</v>
@@ -35990,28 +35999,28 @@
         <v>48</v>
       </c>
       <c r="J27" s="45" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="K27" s="45"/>
       <c r="L27" s="45"/>
     </row>
     <row r="28" customHeight="1" spans="1:12">
       <c r="A28" s="45" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="B28" s="45" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="C28" s="45" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="D28" s="46" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E28" s="47"/>
       <c r="F28" s="47"/>
       <c r="G28" s="58" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="H28" s="49">
         <v>46151</v>
@@ -36020,28 +36029,28 @@
         <v>48</v>
       </c>
       <c r="J28" s="45" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="K28" s="45"/>
       <c r="L28" s="45"/>
     </row>
     <row r="29" customHeight="1" spans="1:12">
       <c r="A29" s="45" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="B29" s="45" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="C29" s="45" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="D29" s="46" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="E29" s="47"/>
       <c r="F29" s="47"/>
       <c r="G29" s="58" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="H29" s="49">
         <v>46151</v>
@@ -36050,28 +36059,28 @@
         <v>48</v>
       </c>
       <c r="J29" s="45" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="K29" s="45"/>
       <c r="L29" s="45"/>
     </row>
     <row r="30" customHeight="1" spans="1:12">
       <c r="A30" s="45" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B30" s="45" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="C30" s="45" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="D30" s="46" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="E30" s="47"/>
       <c r="F30" s="47"/>
       <c r="G30" s="58" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="H30" s="49">
         <v>46151</v>
@@ -36080,17 +36089,14 @@
         <v>50</v>
       </c>
       <c r="J30" s="45" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="K30" s="45" t="s">
         <v>48</v>
       </c>
       <c r="L30" s="58" t="s">
-        <v>523</v>
-      </c>
-    </row>
-    <row r="33" customHeight="1" spans="1:1">
-      <c r="A33" s="56"/>
+        <v>524</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="17">
@@ -36128,14 +36134,15 @@
     <hyperlink ref="G21" r:id="rId13" display="TCAPIPro9.png"/>
     <hyperlink ref="L21" r:id="rId14" display="TCAPIPro9SauRetest.png"/>
     <hyperlink ref="G22" r:id="rId15" display="TCAPIPro10.png"/>
-    <hyperlink ref="G24" r:id="rId16" display="TCAPIPro11.png"/>
-    <hyperlink ref="G25" r:id="rId17" display="TCAPIPro12.png"/>
-    <hyperlink ref="G26" r:id="rId18" display="TCAPIPro13.png"/>
-    <hyperlink ref="G27" r:id="rId19" display="TCAPIPro14.png"/>
-    <hyperlink ref="G28" r:id="rId20" display="TCAPIPro15.png"/>
-    <hyperlink ref="G29" r:id="rId21" display="TCAPIPro16.png"/>
-    <hyperlink ref="G30" r:id="rId22" display="TCAPIPro17.png"/>
-    <hyperlink ref="L30" r:id="rId23" display="TCAPIPro17SauRetest.png"/>
+    <hyperlink ref="L22" r:id="rId16" display="TCAPIPro10SauRetest.png"/>
+    <hyperlink ref="G24" r:id="rId17" display="TCAPIPro11.png"/>
+    <hyperlink ref="G25" r:id="rId18" display="TCAPIPro12.png"/>
+    <hyperlink ref="G26" r:id="rId19" display="TCAPIPro13.png"/>
+    <hyperlink ref="G27" r:id="rId20" display="TCAPIPro14.png"/>
+    <hyperlink ref="G28" r:id="rId21" display="TCAPIPro15.png"/>
+    <hyperlink ref="G29" r:id="rId22" display="TCAPIPro16.png"/>
+    <hyperlink ref="G30" r:id="rId23" display="TCAPIPro17.png"/>
+    <hyperlink ref="L30" r:id="rId24" display="TCAPIPro17SauRetest.png"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
@@ -36150,7 +36157,6 @@
   <dimension ref="A1:L32"/>
   <sheetFormatPr defaultColWidth="12.6296296296296" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="18.3333333333333" customWidth="1"/>
     <col min="2" max="2" width="45.25" customWidth="1"/>
     <col min="3" max="3" width="64.6296296296296" customWidth="1"/>
     <col min="4" max="4" width="30.1296296296296" customWidth="1"/>
@@ -36222,7 +36228,7 @@
         <v>46</v>
       </c>
       <c r="B5" s="24" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="C5" s="25"/>
       <c r="D5" s="26"/>
@@ -36363,21 +36369,21 @@
     </row>
     <row r="13" customHeight="1" spans="1:12">
       <c r="A13" s="45" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="B13" s="45" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="C13" s="45" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="D13" s="46" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="E13" s="47"/>
       <c r="F13" s="47"/>
       <c r="G13" s="48" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="H13" s="49">
         <v>46152</v>
@@ -36386,28 +36392,28 @@
         <v>48</v>
       </c>
       <c r="J13" s="50" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="K13" s="50"/>
       <c r="L13" s="50"/>
     </row>
     <row r="14" customHeight="1" spans="1:12">
       <c r="A14" s="45" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B14" s="45" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="C14" s="45" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="D14" s="46" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="E14" s="47"/>
       <c r="F14" s="47"/>
       <c r="G14" s="48" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="H14" s="49">
         <v>46152</v>
@@ -36416,28 +36422,28 @@
         <v>48</v>
       </c>
       <c r="J14" s="50" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="K14" s="50"/>
       <c r="L14" s="50"/>
     </row>
     <row r="15" customHeight="1" spans="1:12">
       <c r="A15" s="45" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="B15" s="45" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="C15" s="45" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="D15" s="46" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="E15" s="47"/>
       <c r="F15" s="47"/>
       <c r="G15" s="48" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="H15" s="49">
         <v>46152</v>
@@ -36446,14 +36452,14 @@
         <v>48</v>
       </c>
       <c r="J15" s="50" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="K15" s="50"/>
       <c r="L15" s="50"/>
     </row>
     <row r="16" customHeight="1" spans="1:12">
       <c r="A16" s="44" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B16" s="25"/>
       <c r="C16" s="25"/>
@@ -36469,21 +36475,21 @@
     </row>
     <row r="17" customHeight="1" spans="1:12">
       <c r="A17" s="45" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="B17" s="45" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="C17" s="50" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="D17" s="46" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="E17" s="47"/>
       <c r="F17" s="47"/>
       <c r="G17" s="48" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="H17" s="49">
         <v>46136</v>
@@ -36492,32 +36498,32 @@
         <v>50</v>
       </c>
       <c r="J17" s="50" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="K17" s="50" t="s">
         <v>48</v>
       </c>
       <c r="L17" s="48" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
     </row>
     <row r="18" customHeight="1" spans="1:12">
       <c r="A18" s="45" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="B18" s="45" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="C18" s="45" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="D18" s="46" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="E18" s="47"/>
       <c r="F18" s="47"/>
       <c r="G18" s="48" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="H18" s="49">
         <v>46152</v>
@@ -36526,28 +36532,28 @@
         <v>48</v>
       </c>
       <c r="J18" s="50" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="K18" s="50"/>
       <c r="L18" s="50"/>
     </row>
     <row r="19" customHeight="1" spans="1:12">
       <c r="A19" s="45" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="B19" s="45" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="C19" s="51" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="D19" s="46" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="E19" s="47"/>
       <c r="F19" s="47"/>
       <c r="G19" s="48" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="H19" s="49">
         <v>46152</v>
@@ -36556,28 +36562,28 @@
         <v>48</v>
       </c>
       <c r="J19" s="50" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="K19" s="50"/>
       <c r="L19" s="50"/>
     </row>
     <row r="20" customHeight="1" spans="1:12">
       <c r="A20" s="45" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="B20" s="45" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="C20" s="45" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="D20" s="46" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="E20" s="47"/>
       <c r="F20" s="47"/>
       <c r="G20" s="48" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="H20" s="49">
         <v>46152</v>
@@ -36586,28 +36592,28 @@
         <v>48</v>
       </c>
       <c r="J20" s="50" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="K20" s="50"/>
       <c r="L20" s="50"/>
     </row>
     <row r="21" customHeight="1" spans="1:12">
       <c r="A21" s="45" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="B21" s="45" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="C21" s="45" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="D21" s="46" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="E21" s="47"/>
       <c r="F21" s="47"/>
       <c r="G21" s="48" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="H21" s="49">
         <v>46152</v>
@@ -36616,28 +36622,28 @@
         <v>48</v>
       </c>
       <c r="J21" s="50" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="K21" s="50"/>
       <c r="L21" s="50"/>
     </row>
     <row r="22" customHeight="1" spans="1:12">
       <c r="A22" s="45" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="B22" s="45" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="C22" s="45" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="D22" s="46" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="E22" s="47"/>
       <c r="F22" s="47"/>
       <c r="G22" s="48" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="H22" s="49">
         <v>46152</v>
@@ -36646,14 +36652,14 @@
         <v>48</v>
       </c>
       <c r="J22" s="50" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="K22" s="50"/>
       <c r="L22" s="50"/>
     </row>
     <row r="23" customHeight="1" spans="1:12">
       <c r="A23" s="44" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="B23" s="25"/>
       <c r="C23" s="25"/>
@@ -36669,21 +36675,21 @@
     </row>
     <row r="24" customHeight="1" spans="1:12">
       <c r="A24" s="45" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="B24" s="45" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="C24" s="45" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="D24" s="46" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="E24" s="47"/>
       <c r="F24" s="47"/>
       <c r="G24" s="48" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="H24" s="49">
         <v>46152</v>
@@ -36692,28 +36698,28 @@
         <v>48</v>
       </c>
       <c r="J24" s="50" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="K24" s="50"/>
       <c r="L24" s="50"/>
     </row>
     <row r="25" customHeight="1" spans="1:12">
       <c r="A25" s="45" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="B25" s="45" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="C25" s="45" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="D25" s="46" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="E25" s="47"/>
       <c r="F25" s="47"/>
       <c r="G25" s="48" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="H25" s="49">
         <v>46152</v>
@@ -36722,14 +36728,14 @@
         <v>48</v>
       </c>
       <c r="J25" s="50" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="K25" s="50"/>
       <c r="L25" s="50"/>
     </row>
     <row r="26" customHeight="1" spans="1:12">
       <c r="A26" s="44" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="B26" s="25"/>
       <c r="C26" s="25"/>
@@ -36745,21 +36751,21 @@
     </row>
     <row r="27" customHeight="1" spans="1:12">
       <c r="A27" s="45" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="B27" s="45" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="C27" s="50" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="D27" s="46" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="E27" s="47"/>
       <c r="F27" s="52"/>
       <c r="G27" s="53" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="H27" s="49">
         <v>46152</v>
@@ -36768,28 +36774,28 @@
         <v>48</v>
       </c>
       <c r="J27" s="50" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="K27" s="50"/>
       <c r="L27" s="50"/>
     </row>
     <row r="28" customHeight="1" spans="1:12">
       <c r="A28" s="45" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="B28" s="45" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="C28" s="45" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="D28" s="46" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="E28" s="47"/>
       <c r="F28" s="47"/>
       <c r="G28" s="48" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="H28" s="49">
         <v>46152</v>
@@ -36798,28 +36804,28 @@
         <v>48</v>
       </c>
       <c r="J28" s="50" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="K28" s="50"/>
       <c r="L28" s="50"/>
     </row>
     <row r="29" customHeight="1" spans="1:12">
       <c r="A29" s="45" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="B29" s="45" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="C29" s="45" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="D29" s="46" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="E29" s="47"/>
       <c r="F29" s="47"/>
       <c r="G29" s="48" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="H29" s="49">
         <v>46152</v>
@@ -36828,28 +36834,28 @@
         <v>48</v>
       </c>
       <c r="J29" s="50" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="K29" s="50"/>
       <c r="L29" s="50"/>
     </row>
     <row r="30" customHeight="1" spans="1:12">
       <c r="A30" s="45" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="B30" s="45" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="C30" s="45" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="D30" s="46" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="E30" s="47"/>
       <c r="F30" s="47"/>
       <c r="G30" s="48" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="H30" s="49">
         <v>46152</v>
@@ -36858,28 +36864,28 @@
         <v>48</v>
       </c>
       <c r="J30" s="50" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="K30" s="50"/>
       <c r="L30" s="50"/>
     </row>
     <row r="31" customHeight="1" spans="1:12">
       <c r="A31" s="45" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="B31" s="45" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="C31" s="45" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="D31" s="46" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="E31" s="47"/>
       <c r="F31" s="47"/>
       <c r="G31" s="48" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="H31" s="49">
         <v>46152</v>
@@ -36888,28 +36894,28 @@
         <v>48</v>
       </c>
       <c r="J31" s="50" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="K31" s="50"/>
       <c r="L31" s="50"/>
     </row>
     <row r="32" customHeight="1" spans="1:12">
       <c r="A32" s="45" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B32" s="45" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="C32" s="45" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="D32" s="46" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="E32" s="47"/>
       <c r="F32" s="47"/>
       <c r="G32" s="48" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="H32" s="49">
         <v>46152</v>
@@ -36918,7 +36924,7 @@
         <v>48</v>
       </c>
       <c r="J32" s="50" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="K32" s="50"/>
       <c r="L32" s="50"/>

</xml_diff>